<commit_message>
docs(review1): polish and restructure teacher feedback notes in AI_Capstone_Review123_Template.xlsx
</commit_message>
<xml_diff>
--- a/AI_Capstone_Review123_Template.xlsx
+++ b/AI_Capstone_Review123_Template.xlsx
@@ -1,512 +1,247 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22188" windowHeight="8676" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Review1" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Review2" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="Review3" sheetId="3" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr/>
-  <extLst>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="HJhsya24RlBTJwkkSFFv1D69KdXNxYIS7qOfc6pX6uc="/>
-    </ext>
-  </extLst>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="68">
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Mã ĐATN</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Tên ĐATN</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Mã ĐATN</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Tên ĐATN</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Giảng viên Review</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> : </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Thời gian</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>:</t>
-    </r>
-  </si>
-  <si>
-    <t>Tiêu chí</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Giảng viên Review</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-  </si>
-  <si>
-    <t>Gợi ý đánh giá/nhận xét</t>
-  </si>
-  <si>
-    <t>Góp ý/nhận xét của GV Review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Những thay đổi sau lần Review1 </t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Thời gian</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>:</t>
-    </r>
-  </si>
-  <si>
-    <t>Những thay đổi sau lần Review1 là gì ?
-Phản hồi sau lần review 1 từ nhóm ĐATN là gì ?</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Tên ĐATN</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> :</t>
-    </r>
-  </si>
-  <si>
-    <t>Quản trị dự án/lập kế hoạch</t>
-  </si>
-  <si>
-    <t>Email các GV review</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Giảng viên Review</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> : </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Thời gian</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>:</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Mục tiêu của đề tài (problem) </t>
-  </si>
-  <si>
-    <t>Những thay đổi sau lần Review2</t>
-  </si>
-  <si>
-    <t>Lập kế hoạch có đầy đủ không ?</t>
-  </si>
-  <si>
-    <t>Những thay đổi sau lần Review2 là gì ?
-Phản hồi sau lần review 2 từ nhóm ĐATN là gì ?</t>
-  </si>
-  <si>
-    <t>Phát biểu bài toán có đủ rõ ràng hay không ?</t>
-  </si>
-  <si>
-    <t>Phương pháp/mô hình quản trị dự án/công cụ hỗ trợ quản trị ?</t>
-  </si>
-  <si>
-    <t>Các phương pháp/hướng tiếp cận / mô hình giải quyết vấn đề đã đặt ra trong ĐATN</t>
-  </si>
-  <si>
-    <t>Nguyễn Trọng Tài</t>
-  </si>
-  <si>
-    <t>taint51@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Đánh giá kết quả của các phương pháp/hướng tiếp cận / mô hình giải đã đặt ra trong ĐATN</t>
-  </si>
-  <si>
-    <t>Hướng tiếp cận 1</t>
-  </si>
-  <si>
-    <t>Kết quả cuối cùng là gi ? (proposed solution) 
-Kết quả mong muốn phải đạt được của đề tài là gì ?</t>
-  </si>
-  <si>
-    <t>Phương pháp thu thập dữ liệu/chuẩn bị dữ liệu là gì ?</t>
-  </si>
-  <si>
-    <t>Chọn lựa mô hình nào , các đặc trưng gì ? Như thế nào ?
-Thiết kế thành phần biểu diễn dữ liệu như thế nào ?
-Thuật toán gì ? Thiết kế ra sao ?</t>
-  </si>
-  <si>
-    <t>Báo cáo khoa học/paper</t>
-  </si>
-  <si>
-    <t>Huấn luyện / đánh giá mô hình như thế nào ?
-Độ phức tạp thuật toán như thế nào ?</t>
-  </si>
-  <si>
-    <t>Lê Phú Nguyên</t>
-  </si>
-  <si>
-    <t>Tinh chỉnh các tham số như thế nào ?
-Cải tiến gì trong thuật toán ?</t>
-  </si>
-  <si>
-    <t>Khác</t>
-  </si>
-  <si>
-    <t>Hướng tiếp cận 2</t>
-  </si>
-  <si>
-    <t>nguyenlp9@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Software hoàn chỉnh</t>
-  </si>
-  <si>
-    <t>Nguyễn Quốc Trung</t>
-  </si>
-  <si>
-    <t>TrungNQ46@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Software prototype</t>
-  </si>
-  <si>
-    <t>Hướng tiếp cận 3</t>
-  </si>
-  <si>
-    <t>Nguyễn Hồng Hải</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HaiNH51@fe.edu.vn </t>
-  </si>
-  <si>
-    <t>Framework/platform/library API</t>
-  </si>
-  <si>
-    <t>Vũ Hà Anh</t>
-  </si>
-  <si>
-    <t>AnhVH54@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Nguyễn Xuân Huy</t>
-  </si>
-  <si>
-    <t>huynx23@fe.edu.vn</t>
-  </si>
-  <si>
-    <t>Tính khả thi
-Xác định scope của đề tài</t>
-  </si>
-  <si>
-    <t>Dựa trên hướng tiếp cận nào; phương pháp/thuật toán/mô hình nào ==&gt; số lượng tìm hiểu là bao nhiêu ?</t>
-  </si>
-  <si>
-    <t>Dự kiến triển khai từ đầu hay tái sử dụng lại API/Framework/Platform có sẵn ?</t>
-  </si>
-  <si>
-    <t>Có cải tiến hay đưa ra mô hình, thuật toán mới không ? Số lượng là bao nhiêu ?</t>
-  </si>
-  <si>
-    <t>Tập dữ liệu mẫu tự xây dựng hay có sẵn ? Có thay đổi gì trên tập dữ liệu có sẵn hay không ?</t>
-  </si>
-  <si>
-    <t>So sánh các phương pháp/ thảo luận / kết luận</t>
-  </si>
-  <si>
-    <t>Giá trị của đề tài</t>
-  </si>
-  <si>
-    <t>Đề tài có tính thực tế không ? Có thể vận dụng được trong thực tế hay không ?</t>
-  </si>
-  <si>
-    <t>Đề tài có ý nghĩa không (có giá trị, ý nghĩa khoa học hay không, nếu là báo cáo khoa học) ?</t>
-  </si>
-  <si>
-    <t>Đề tài có mới ?có  sáng tạo không ?</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <i/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-        <u/>
-      </rPr>
-      <t>Nhận xét chung của GV_</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve"> : 
-- Hoàn thiện report
-- Bổ sung tinh chỉnh models
-- Chỉnh sửa demo
-- Tăng độ chính xác model
-- Khuyến nghị BV lần 1</t>
-    </r>
-  </si>
-  <si>
-    <t>Khuyến nghị của GV Review:</t>
-  </si>
-  <si>
-    <t>Kết quả khuyến nghị</t>
-  </si>
-  <si>
-    <t>1/Kết quả KLTN đủ tiêu chuẩn để bảo vệ lần 1</t>
-  </si>
-  <si>
-    <t>2/Cần cập nhật, bổ sung theo những góp ý của GV Review để bảo vệ lần 1</t>
-  </si>
-  <si>
-    <t>3/Kết quả KLTN còn nhiều thiếu sót. Phải bổ sung đầy đủ theo những góp ý và bảo vệ lần 2</t>
-  </si>
-  <si>
-    <t>4/Kết quả KLTN có những thiếu sót nghiêm trọng, không đáp ứng được tiêu chuẩn của KLTN ngành TTNT. Nhóm nên chấm dứt dự án KLTN</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="29">
     <font>
-      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font/>
-    <font>
-      <sz val="11.0"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="11.0"/>
-      <color theme="1"/>
       <name val="Calibri"/>
+      <charset val="134"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <u/>
-      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <i val="1"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <i val="1"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b/>
-      <i/>
-      <sz val="11.0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <i val="1"/>
       <color rgb="FFFF0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FF1F1F1F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -514,9 +249,201 @@
         <bgColor rgb="FFFFC000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
-    <border/>
+  <borders count="19">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -530,6 +457,7 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -541,12 +469,8 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -555,30 +479,38 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -588,6 +520,7 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -596,116 +529,711 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="13" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="14" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+  <cellXfs count="41">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf quotePrefix="1" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="9" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="17">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color theme="4"/>
+        </left>
+        <right style="thin">
+          <color theme="4"/>
+        </right>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <horizontal style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    </tableStyle>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -895,190 +1423,335 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <dimension ref="B2:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.71"/>
-    <col customWidth="1" min="2" max="2" width="47.57"/>
-    <col customWidth="1" min="3" max="3" width="49.71"/>
-    <col customWidth="1" min="4" max="4" width="86.14"/>
-    <col customWidth="1" min="5" max="5" width="26.71"/>
-    <col customWidth="1" min="6" max="6" width="20.57"/>
-    <col customWidth="1" min="7" max="7" width="19.86"/>
-    <col customWidth="1" min="8" max="26" width="8.71"/>
+    <col width="8.71296296296296" customWidth="1" min="1" max="1"/>
+    <col width="47.5740740740741" customWidth="1" min="2" max="2"/>
+    <col width="49.712962962963" customWidth="1" min="3" max="3"/>
+    <col width="92" customWidth="1" style="25" min="4" max="4"/>
+    <col width="26.712962962963" customWidth="1" min="5" max="5"/>
+    <col width="20.5740740740741" customWidth="1" min="6" max="6"/>
+    <col width="19.8611111111111" customWidth="1" min="7" max="7"/>
+    <col width="8.71296296296296" customWidth="1" min="8" max="26"/>
   </cols>
   <sheetData>
+    <row r="2"/>
     <row r="3">
-      <c r="B3" s="2" t="s">
-        <v>1</v>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Tên ĐATN : Hệ thống phát hiện vi phạm mũ bảo hộ lao động theo thời gian thực trong môi trường công trường xây dựng dựa trên kiến trúc Rep-YOLO11s</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="2" t="s">
-        <v>7</v>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Giảng viên Review : Hội đồng GV Review ĐATN (Thầy Nguyễn Trọng Tài, Thầy Lê Phú Nguyên, Thầy Nguyễn Quốc Trung, Thầy Nguyễn Hồng Hải, Cô Vũ Hà Anh, Thầy Nguyễn Xuân Huy)</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="2" t="s">
-        <v>11</v>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Thời gian: Học kỳ Fall 2026 - Đợt Review 1</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1">
-      <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="8"/>
-    </row>
-    <row r="8" ht="34.5" customHeight="1">
-      <c r="B8" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="14"/>
-      <c r="F8" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" ht="34.5" customHeight="1">
-      <c r="B9" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="14"/>
-      <c r="F9" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="G9" s="20" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" ht="34.5" customHeight="1">
-      <c r="B10" s="19"/>
-      <c r="C10" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" s="14"/>
-      <c r="F10" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" ht="34.5" customHeight="1">
-      <c r="B11" s="19"/>
-      <c r="C11" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="14"/>
-      <c r="F11" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" ht="34.5" customHeight="1">
-      <c r="B12" s="19"/>
-      <c r="C12" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D12" s="14"/>
-      <c r="F12" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="G12" s="22" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="13"/>
-      <c r="C13" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="14"/>
-      <c r="F13" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" ht="34.5" customHeight="1">
-      <c r="B14" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14" s="14"/>
-    </row>
-    <row r="15" ht="34.5" customHeight="1">
-      <c r="B15" s="19"/>
-      <c r="C15" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="14"/>
-    </row>
-    <row r="16" ht="34.5" customHeight="1">
-      <c r="B16" s="19"/>
-      <c r="C16" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" s="14"/>
-    </row>
-    <row r="17" ht="34.5" customHeight="1">
-      <c r="B17" s="13"/>
-      <c r="C17" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="14"/>
-    </row>
-    <row r="18" ht="34.5" customHeight="1">
-      <c r="B18" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="14"/>
-    </row>
-    <row r="19" ht="34.5" customHeight="1">
-      <c r="B19" s="19"/>
-      <c r="C19" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="D19" s="14"/>
-    </row>
-    <row r="20" ht="34.5" customHeight="1">
-      <c r="B20" s="13"/>
-      <c r="C20" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="14"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Tiêu chí</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Gợi ý đánh giá/nhận xét</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Góp ý/nhận xét của GV Review</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>Email các GV review</t>
+        </is>
+      </c>
+      <c r="G7" s="32" t="n"/>
+    </row>
+    <row r="8" ht="153" customHeight="1">
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mục tiêu của đề tài (problem) </t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Phát biểu bài toán có đủ rõ ràng hay không ?</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>- Cần phát biểu bài toán rõ ràng, cụ thể và định lượng: Xác định rõ mục tiêu là phát hiện công nhân tuân thủ đội mũ / không đội mũ bảo hộ lao động theo thời gian thực từ camera giám sát công trường (CCTV).
+- Làm rõ kịch bản đầu ra nghiệp vụ: Khi phát hiện vi phạm (không đội mũ), hệ thống cần gửi tín hiệu/thông tin cảnh báo tức thời về thiết bị giám sát của người quản lý an toàn công trường.
+- Gợi ý mở rộng (nếu khả thi): Xem xét khả năng phân loại thêm màu sắc của mũ bảo hộ (trắng, vàng, đỏ, xanh...) để phân biệt chức danh/vị trí làm việc của công nhân và kỹ sư.</t>
+        </is>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>Nguyễn Trọng Tài</t>
+        </is>
+      </c>
+      <c r="G8" s="32" t="inlineStr">
+        <is>
+          <t>taint51@fe.edu.vn</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="102" customHeight="1">
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Kết quả cuối cùng là gi ? (proposed solution) 
+Kết quả mong muốn phải đạt được của đề tài là gì ?</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="inlineStr">
+        <is>
+          <t>Báo cáo khoa học/paper</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>- Báo cáo khoa học/paper cần có cấu trúc chuẩn mực học thuật: Trình bày rõ ràng phương pháp nghiên cứu (Methodology), cơ sở lý thuyết của các cải tiến, và thiết kế thực nghiệm bài bản.
+- Phải có bảng đối chuẩn thực nghiệm chi tiết giữa mô hình đề xuất với các mô hình baseline (YOLO11s, YOLOv8s) theo các chỉ số khoa học: mAP50, mAP50-95, Recall, độ trễ (latency), FPS và số lượng tham số (Params, FLOPs).</t>
+        </is>
+      </c>
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>Lê Phú Nguyên</t>
+        </is>
+      </c>
+      <c r="G9" s="32" t="inlineStr">
+        <is>
+          <t>nguyenlp9@fe.edu.vn</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="102" customHeight="1">
+      <c r="B10" s="36" t="n"/>
+      <c r="C10" s="34" t="inlineStr">
+        <is>
+          <t>Software hoàn chỉnh</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>- Cần xác định rõ môi trường triển khai thực tế của phần mềm: Hệ thống chạy trên máy chủ giám sát trung tâm, máy trạm PC có GPU hay thiết bị biên tại công trường?
+- Làm rõ luồng chức năng đầu ra (Output): Hiển thị bounding box nhận diện theo thời gian thực từ luồng RTSP camera, đồng thời có cơ chế ghi nhận log vi phạm và gửi thông báo cảnh báo về giao diện quản lý.</t>
+        </is>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
+        <is>
+          <t>Nguyễn Quốc Trung</t>
+        </is>
+      </c>
+      <c r="G10" s="32" t="inlineStr">
+        <is>
+          <t>TrungNQ46@fe.edu.vn</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="102" customHeight="1">
+      <c r="B11" s="36" t="n"/>
+      <c r="C11" s="34" t="inlineStr">
+        <is>
+          <t>Software prototype</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>- Bản prototype cần chứng minh được luồng xử lý hoàn chỉnh (End-to-End pipeline): Nhận luồng video đầu vào -&gt; Tiền xử lý -&gt; Mô hình suy luận (Inference) -&gt; Xuất kết quả phát hiện trực quan.
+- Cần phân tích rõ mô hình baseline giải quyết được bài toán đến mức độ nào, những hạn chế còn tồn tại và mô hình đề xuất cải thiện được những điểm nghẽn cụ thể nào.</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>Nguyễn Hồng Hải</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HaiNH51@fe.edu.vn </t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="85" customHeight="1">
+      <c r="B12" s="36" t="n"/>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>Framework/platform/library API</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>- Nêu rõ các framework, thư viện và nền tảng sử dụng: PyTorch, Ultralytics YOLO, OpenCV, cùng các công cụ tối ưu hóa suy luận (ONNX Runtime, TensorRT).
+- Về dữ liệu: Đối với hướng mở rộng phân loại màu mũ, cần bổ sung tập dữ liệu có gán nhãn đa lớp màu sắc tương ứng; ở phạm vi hiện tại cần chuẩn hóa API dữ liệu đầu vào/đầu ra rõ ràng.</t>
+        </is>
+      </c>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>Vũ Hà Anh</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>AnhVH54@fe.edu.vn</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="B13" s="37" t="n"/>
+      <c r="C13" s="34" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="inlineStr">
+        <is>
+          <t>- Hoàn thiện mã nguồn chuẩn hóa, đóng gói dạng module rõ ràng, có tài liệu hướng dẫn cài đặt và tái lập thực nghiệm (Reproducibility) trên GitHub.</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>Nguyễn Xuân Huy</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>huynx23@fe.edu.vn</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="153" customHeight="1">
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>Tính khả thi
+Xác định scope của đề tài</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Dựa trên hướng tiếp cận nào; phương pháp/thuật toán/mô hình nào ==&gt; số lượng tìm hiểu là bao nhiêu ?</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>- Định vị học thuật rõ ràng: Đề tài thuộc nhánh Deep Learning / Computer Vision, giải quyết bài toán Phát hiện đối tượng (Object Detection) dựa trên họ mô hình YOLO (Single-Stage Detector); khẳng định rõ không phải bài toán Phân vùng ảnh (Segmentation).
+- Yêu cầu vẽ lại sơ đồ kiến trúc chi tiết: Thể hiện rõ các khối mô-đun cải tiến và luồng dữ liệu.
+- Kế hoạch cho Review 2: Phải chạy thực nghiệm đối chuẩn đầy đủ giữa Baseline 1 (YOLO11s) và Baseline 2 (YOLOv8s) với các phương pháp cải tiến, phân tích và đánh giá định lượng xem phương pháp nào phù hợp nhất trước khi đưa ra kết luận.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="102" customHeight="1">
+      <c r="B15" s="36" t="n"/>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Dự kiến triển khai từ đầu hay tái sử dụng lại API/Framework/Platform có sẵn ?</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>- Xây dựng Roadmap (lộ trình thực hiện) chi tiết, rõ ràng qua từng cột mốc Review 1 -&gt; Review 2 -&gt; Review 3 -&gt; Bảo vệ tốt nghiệp.
+- Phân định rõ phạm vi: Phần nào tái sử dụng (pre-trained backbone từ COCO, thư viện Ultralytics, tập dữ liệu SHWD/VOC2028), phần nào do nhóm tự nghiên cứu thiết kế mới (tự viết và tích hợp 4 module cải tiến kiến trúc và hàm mất mát tùy biến).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="136" customHeight="1">
+      <c r="B16" s="36" t="n"/>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Có cải tiến hay đưa ra mô hình, thuật toán mới không ? Số lượng là bao nhiêu ?</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>- Nhóm đề xuất mô hình cải tiến Rep-YOLO11s gồm 4 module trọng tâm: (1) CoordConv ở tầng Stem, (2) RepConv ở Backbone, (3) BiFormer Attention ở Neck, (4) Focal-EIoU ở Head.
+- Phải giải thích rõ mục đích của từng module: CoordConv khử báo động sàn, RepConv tối ưu tốc độ suy luận, BiFormer lọc bụi và lóa sáng, Focal-EIoU bắt mũ nhỏ ở cự ly xa.
+- Yêu cầu thực hiện Ablation Study (nghiên cứu bóc tách A0 -&gt; A6) ở Review 2 để chứng minh đóng góp của từng cải tiến.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="85" customHeight="1">
+      <c r="B17" s="37" t="n"/>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Tập dữ liệu mẫu tự xây dựng hay có sẵn ? Có thay đổi gì trên tập dữ liệu có sẵn hay không ?</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>- Sử dụng tập dữ liệu chuẩn SHWD/VOC2028 gồm 7,581 ảnh authentic, làm rõ vấn đề mất cân bằng dữ liệu nghiêm trọng giữa 2 lớp (tỷ lệ 1:12 giữa hat và person).
+- Nêu rõ giải pháp xử lý mất cân bằng: Sử dụng Alpha-Balanced Focal Loss tại Head kết hợp cơ chế gán nhãn TAL và kỹ thuật tăng cường dữ liệu đặc thù công trường (Mosaic, biến đổi bóng đổ, lóa sáng, khói bụi).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="68" customHeight="1">
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>Giá trị của đề tài</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Đề tài có tính thực tế không ? Có thể vận dụng được trong thực tế hay không ?</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="inlineStr">
+        <is>
+          <t>- Đề tài có tính ứng dụng thực tiễn rất cao, đáp ứng nhu cầu cấp thiết về tự động hóa giám sát an toàn lao động tại các công trình xây dựng và nhà máy.
+- Cần đặc biệt chú trọng tính khả thi triển khai: Tốc độ xử lý phải đạt thời gian thực (&gt;= 30 FPS) trên hệ thống camera giám sát thông thường.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="102" customHeight="1">
+      <c r="B19" s="36" t="n"/>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Đề tài có ý nghĩa không (có giá trị, ý nghĩa khoa học hay không, nếu là báo cáo khoa học) ?</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>- Có ý nghĩa khoa học rõ ràng trong việc giải quyết các thách thức đặc thù của thị giác máy tính trong môi trường khắc nghiệt: Nhận diện vật thể nhỏ, che khuất, triệt tiêu báo động giả và cân bằng tối ưu giữa độ chính xác và độ trễ tính toán.
+- Kết quả nghiên cứu có giá trị đóng góp thành báo cáo khoa học chuẩn mực sẵn sàng nghiệm thu và công bố.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="85" customHeight="1">
+      <c r="B20" s="37" t="n"/>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Đề tài có mới ?có  sáng tạo không ?</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="inlineStr">
+        <is>
+          <t>- Tính mới và sáng tạo thể hiện ở việc tiên phong tích hợp kỹ thuật tái tham số hóa cấu trúc (RepConv) và chú ý định tuyến thưa 2 cấp (BiFormer) vào kiến trúc thế hệ mới nhất YOLO11s.
+- Đề xuất giải pháp nhúng tọa độ không gian (CoordConv) phá vỡ tính bất biến tịnh tiến để giải quyết triệt để lỗi đặc thù của camera quan sát góc cao.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -2062,210 +2735,285 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B14:B17"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B9:B13"/>
-    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B2:D2"/>
     <mergeCell ref="B18:B20"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="portrait" paperSize="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <dimension ref="B2:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.71"/>
-    <col customWidth="1" min="2" max="2" width="47.57"/>
-    <col customWidth="1" min="3" max="3" width="57.86"/>
-    <col customWidth="1" min="4" max="4" width="93.29"/>
-    <col customWidth="1" min="5" max="5" width="26.71"/>
-    <col customWidth="1" min="6" max="6" width="20.57"/>
-    <col customWidth="1" min="7" max="26" width="8.71"/>
+    <col width="8.71296296296296" customWidth="1" min="1" max="1"/>
+    <col width="47.5740740740741" customWidth="1" min="2" max="2"/>
+    <col width="57.8611111111111" customWidth="1" min="3" max="3"/>
+    <col width="93.287037037037" customWidth="1" min="4" max="4"/>
+    <col width="26.712962962963" customWidth="1" min="5" max="5"/>
+    <col width="20.5740740740741" customWidth="1" min="6" max="6"/>
+    <col width="8.71296296296296" customWidth="1" min="7" max="26"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="1" t="s">
-        <v>5</v>
+    <row r="2" ht="14.4" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Mã ĐATN :</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="14.4" customHeight="1">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Tên ĐATN :</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="14.4" customHeight="1">
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giảng viên Review : </t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="14.4" customHeight="1">
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Thời gian:</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1">
-      <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>9</v>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Tiêu chí</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Gợi ý đánh giá/nhận xét</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Góp ý/nhận xét của GV Review</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="31.5" customHeight="1">
-      <c r="B8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="6"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Những thay đổi sau lần Review1 </t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Những thay đổi sau lần Review1 là gì ?
+Phản hồi sau lần review 1 từ nhóm ĐATN là gì ?</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n"/>
     </row>
     <row r="9" ht="31.5" customHeight="1">
-      <c r="B9" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="6"/>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Quản trị dự án/lập kế hoạch</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Lập kế hoạch có đầy đủ không ?</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n"/>
     </row>
     <row r="10" ht="31.5" customHeight="1">
-      <c r="B10" s="13"/>
-      <c r="C10" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="6"/>
+      <c r="B10" s="37" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Phương pháp/mô hình quản trị dự án/công cụ hỗ trợ quản trị ?</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n"/>
     </row>
     <row r="11" ht="31.5" customHeight="1">
-      <c r="B11" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="14"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="19"/>
-      <c r="C13" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="14"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="19"/>
-      <c r="C14" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="14"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="19"/>
-      <c r="C15" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="14"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="13"/>
-      <c r="C16" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="14"/>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Các phương pháp/hướng tiếp cận / mô hình giải quyết vấn đề đã đặt ra trong ĐATN</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="n"/>
+      <c r="D11" s="39" t="n"/>
+    </row>
+    <row r="12" ht="14.4" customHeight="1">
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Hướng tiếp cận 1</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>Phương pháp thu thập dữ liệu/chuẩn bị dữ liệu là gì ?</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n"/>
+    </row>
+    <row r="13" ht="43.2" customHeight="1">
+      <c r="B13" s="36" t="n"/>
+      <c r="C13" s="34" t="inlineStr">
+        <is>
+          <t>Chọn lựa mô hình nào , các đặc trưng gì ? Như thế nào ?
+Thiết kế thành phần biểu diễn dữ liệu như thế nào ?
+Thuật toán gì ? Thiết kế ra sao ?</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="28.8" customHeight="1">
+      <c r="B14" s="36" t="n"/>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>Huấn luyện / đánh giá mô hình như thế nào ?
+Độ phức tạp thuật toán như thế nào ?</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n"/>
+    </row>
+    <row r="15" ht="28.8" customHeight="1">
+      <c r="B15" s="36" t="n"/>
+      <c r="C15" s="34" t="inlineStr">
+        <is>
+          <t>Tinh chỉnh các tham số như thế nào ?
+Cải tiến gì trong thuật toán ?</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="n"/>
+    </row>
+    <row r="16" ht="14.4" customHeight="1">
+      <c r="B16" s="37" t="n"/>
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="n"/>
     </row>
     <row r="17" ht="48.75" customHeight="1">
-      <c r="B17" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="14"/>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Hướng tiếp cận 2</t>
+        </is>
+      </c>
+      <c r="C17" s="34" t="inlineStr">
+        <is>
+          <t>Phương pháp thu thập dữ liệu/chuẩn bị dữ liệu là gì ?</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="n"/>
     </row>
     <row r="18" ht="48.75" customHeight="1">
-      <c r="B18" s="19"/>
-      <c r="C18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="14"/>
+      <c r="B18" s="36" t="n"/>
+      <c r="C18" s="34" t="inlineStr">
+        <is>
+          <t>Chọn lựa mô hình nào , các đặc trưng gì ? Như thế nào ?
+Thiết kế thành phần biểu diễn dữ liệu như thế nào ?
+Thuật toán gì ? Thiết kế ra sao ?</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n"/>
     </row>
     <row r="19" ht="48.75" customHeight="1">
-      <c r="B19" s="19"/>
-      <c r="C19" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="14"/>
+      <c r="B19" s="36" t="n"/>
+      <c r="C19" s="34" t="inlineStr">
+        <is>
+          <t>Huấn luyện / đánh giá mô hình như thế nào ?
+Độ phức tạp thuật toán như thế nào ?</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n"/>
     </row>
     <row r="20" ht="48.75" customHeight="1">
-      <c r="B20" s="19"/>
-      <c r="C20" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="14"/>
+      <c r="B20" s="36" t="n"/>
+      <c r="C20" s="34" t="inlineStr">
+        <is>
+          <t>Tinh chỉnh các tham số như thế nào ?
+Cải tiến gì trong thuật toán ?</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n"/>
     </row>
     <row r="21" ht="48.75" customHeight="1">
-      <c r="B21" s="13"/>
-      <c r="C21" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="14"/>
+      <c r="B21" s="37" t="n"/>
+      <c r="C21" s="34" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="n"/>
     </row>
     <row r="22" ht="48.75" customHeight="1">
-      <c r="B22" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="14"/>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>Hướng tiếp cận 3</t>
+        </is>
+      </c>
+      <c r="C22" s="34" t="inlineStr">
+        <is>
+          <t>Phương pháp thu thập dữ liệu/chuẩn bị dữ liệu là gì ?</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n"/>
     </row>
     <row r="23" ht="48.75" customHeight="1">
-      <c r="B23" s="19"/>
-      <c r="C23" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="14"/>
+      <c r="B23" s="36" t="n"/>
+      <c r="C23" s="34" t="inlineStr">
+        <is>
+          <t>Chọn lựa mô hình nào , các đặc trưng gì ? Như thế nào ?
+Thiết kế thành phần biểu diễn dữ liệu như thế nào ?
+Thuật toán gì ? Thiết kế ra sao ?</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n"/>
     </row>
     <row r="24" ht="48.75" customHeight="1">
-      <c r="B24" s="19"/>
-      <c r="C24" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="14"/>
+      <c r="B24" s="36" t="n"/>
+      <c r="C24" s="34" t="inlineStr">
+        <is>
+          <t>Huấn luyện / đánh giá mô hình như thế nào ?
+Độ phức tạp thuật toán như thế nào ?</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n"/>
     </row>
     <row r="25" ht="48.75" customHeight="1">
-      <c r="B25" s="19"/>
-      <c r="C25" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="14"/>
+      <c r="B25" s="36" t="n"/>
+      <c r="C25" s="34" t="inlineStr">
+        <is>
+          <t>Tinh chỉnh các tham số như thế nào ?
+Cải tiến gì trong thuật toán ?</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n"/>
     </row>
     <row r="26" ht="48.75" customHeight="1">
-      <c r="B26" s="13"/>
-      <c r="C26" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="14"/>
+      <c r="B26" s="37" t="n"/>
+      <c r="C26" s="34" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1"/>
@@ -3243,285 +3991,381 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
     <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B12:B16"/>
     <mergeCell ref="B22:B26"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:B16"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="portrait" paperSize="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <dimension ref="A2:Z34"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="8.71"/>
-    <col customWidth="1" min="2" max="2" width="66.29"/>
-    <col customWidth="1" min="3" max="3" width="57.86"/>
-    <col customWidth="1" min="4" max="4" width="93.29"/>
-    <col customWidth="1" min="5" max="5" width="26.71"/>
-    <col customWidth="1" min="6" max="6" width="20.57"/>
-    <col customWidth="1" min="7" max="26" width="8.71"/>
+    <col width="8.71296296296296" customWidth="1" min="1" max="1"/>
+    <col width="66.287037037037" customWidth="1" min="2" max="2"/>
+    <col width="57.8611111111111" customWidth="1" min="3" max="3"/>
+    <col width="93.287037037037" customWidth="1" min="4" max="4"/>
+    <col width="26.712962962963" customWidth="1" min="5" max="5"/>
+    <col width="20.5740740740741" customWidth="1" min="6" max="6"/>
+    <col width="8.71296296296296" customWidth="1" min="7" max="26"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="1" t="s">
-        <v>17</v>
+    <row r="2" ht="14.4" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Mã ĐATN :</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="14.4" customHeight="1">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Tên ĐATN :</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="14.4" customHeight="1">
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giảng viên Review : </t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="14.4" customHeight="1">
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Thời gian:</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="31.5" customHeight="1">
-      <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9" ht="31.5" hidden="1" customHeight="1">
-      <c r="B9" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" ht="31.5" hidden="1" customHeight="1">
-      <c r="B10" s="13"/>
-      <c r="C10" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="3"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Tiêu chí</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Gợi ý đánh giá/nhận xét</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Góp ý/nhận xét của GV Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28.8" customHeight="1">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Những thay đổi sau lần Review2</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Những thay đổi sau lần Review2 là gì ?
+Phản hồi sau lần review 2 từ nhóm ĐATN là gì ?</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n"/>
+    </row>
+    <row r="9" hidden="1" ht="31.5" customHeight="1">
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>Quản trị dự án/lập kế hoạch</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Lập kế hoạch có đầy đủ không ?</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n"/>
+    </row>
+    <row r="10" hidden="1" ht="31.5" customHeight="1">
+      <c r="B10" s="37" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Phương pháp/mô hình quản trị dự án/công cụ hỗ trợ quản trị ?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n"/>
     </row>
     <row r="11" ht="31.5" customHeight="1">
-      <c r="B11" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Đánh giá kết quả của các phương pháp/hướng tiếp cận / mô hình giải đã đặt ra trong ĐATN</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="n"/>
+      <c r="D11" s="39" t="n"/>
     </row>
     <row r="12" ht="48.75" customHeight="1">
-      <c r="B12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="14"/>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>Hướng tiếp cận 1</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>Phương pháp thu thập dữ liệu/chuẩn bị dữ liệu là gì ?</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n"/>
     </row>
     <row r="13" ht="48.75" customHeight="1">
-      <c r="B13" s="19"/>
-      <c r="C13" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="14"/>
+      <c r="B13" s="36" t="n"/>
+      <c r="C13" s="34" t="inlineStr">
+        <is>
+          <t>Chọn lựa mô hình nào , các đặc trưng gì ? Như thế nào ?
+Thiết kế thành phần biểu diễn dữ liệu như thế nào ?
+Thuật toán gì ? Thiết kế ra sao ?</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n"/>
     </row>
     <row r="14" ht="48.75" customHeight="1">
-      <c r="B14" s="19"/>
-      <c r="C14" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="14"/>
+      <c r="B14" s="36" t="n"/>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>Huấn luyện / đánh giá mô hình như thế nào ?
+Độ phức tạp thuật toán như thế nào ?</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n"/>
     </row>
     <row r="15" ht="48.75" customHeight="1">
-      <c r="B15" s="19"/>
-      <c r="C15" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="14"/>
+      <c r="B15" s="36" t="n"/>
+      <c r="C15" s="34" t="inlineStr">
+        <is>
+          <t>Tinh chỉnh các tham số như thế nào ?
+Cải tiến gì trong thuật toán ?</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="n"/>
     </row>
     <row r="16" ht="48.75" customHeight="1">
-      <c r="B16" s="13"/>
-      <c r="C16" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="14"/>
+      <c r="B16" s="37" t="n"/>
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="n"/>
     </row>
     <row r="17" ht="48.75" customHeight="1">
-      <c r="B17" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="14"/>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Hướng tiếp cận 2</t>
+        </is>
+      </c>
+      <c r="C17" s="34" t="inlineStr">
+        <is>
+          <t>Phương pháp thu thập dữ liệu/chuẩn bị dữ liệu là gì ?</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="n"/>
     </row>
     <row r="18" ht="48.75" customHeight="1">
-      <c r="B18" s="19"/>
-      <c r="C18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="14"/>
+      <c r="B18" s="36" t="n"/>
+      <c r="C18" s="34" t="inlineStr">
+        <is>
+          <t>Chọn lựa mô hình nào , các đặc trưng gì ? Như thế nào ?
+Thiết kế thành phần biểu diễn dữ liệu như thế nào ?
+Thuật toán gì ? Thiết kế ra sao ?</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n"/>
     </row>
     <row r="19" ht="48.75" customHeight="1">
-      <c r="B19" s="19"/>
-      <c r="C19" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="14"/>
+      <c r="B19" s="36" t="n"/>
+      <c r="C19" s="34" t="inlineStr">
+        <is>
+          <t>Huấn luyện / đánh giá mô hình như thế nào ?
+Độ phức tạp thuật toán như thế nào ?</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n"/>
     </row>
     <row r="20" ht="48.75" customHeight="1">
-      <c r="B20" s="19"/>
-      <c r="C20" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="14"/>
+      <c r="B20" s="36" t="n"/>
+      <c r="C20" s="34" t="inlineStr">
+        <is>
+          <t>Tinh chỉnh các tham số như thế nào ?
+Cải tiến gì trong thuật toán ?</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n"/>
     </row>
     <row r="21" ht="48.75" customHeight="1">
-      <c r="B21" s="13"/>
-      <c r="C21" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="14"/>
+      <c r="B21" s="37" t="n"/>
+      <c r="C21" s="34" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="n"/>
     </row>
     <row r="22" ht="48.75" customHeight="1">
-      <c r="B22" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" s="14"/>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>Hướng tiếp cận 3</t>
+        </is>
+      </c>
+      <c r="C22" s="34" t="inlineStr">
+        <is>
+          <t>Phương pháp thu thập dữ liệu/chuẩn bị dữ liệu là gì ?</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n"/>
     </row>
     <row r="23" ht="48.75" customHeight="1">
-      <c r="B23" s="19"/>
-      <c r="C23" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="14"/>
+      <c r="B23" s="36" t="n"/>
+      <c r="C23" s="34" t="inlineStr">
+        <is>
+          <t>Chọn lựa mô hình nào , các đặc trưng gì ? Như thế nào ?
+Thiết kế thành phần biểu diễn dữ liệu như thế nào ?
+Thuật toán gì ? Thiết kế ra sao ?</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n"/>
     </row>
     <row r="24" ht="48.75" customHeight="1">
-      <c r="B24" s="19"/>
-      <c r="C24" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="14"/>
+      <c r="B24" s="36" t="n"/>
+      <c r="C24" s="34" t="inlineStr">
+        <is>
+          <t>Huấn luyện / đánh giá mô hình như thế nào ?
+Độ phức tạp thuật toán như thế nào ?</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n"/>
     </row>
     <row r="25" ht="48.75" customHeight="1">
-      <c r="B25" s="19"/>
-      <c r="C25" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="14"/>
+      <c r="B25" s="36" t="n"/>
+      <c r="C25" s="34" t="inlineStr">
+        <is>
+          <t>Tinh chỉnh các tham số như thế nào ?
+Cải tiến gì trong thuật toán ?</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n"/>
     </row>
     <row r="26" ht="48.75" customHeight="1">
-      <c r="B26" s="13"/>
-      <c r="C26" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="14"/>
+      <c r="B26" s="37" t="n"/>
+      <c r="C26" s="34" t="inlineStr">
+        <is>
+          <t>Khác</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n"/>
     </row>
     <row r="27" ht="33.75" customHeight="1">
-      <c r="B27" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-    </row>
-    <row r="29" ht="30.0" customHeight="1">
-      <c r="B29" s="26" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="30" ht="30.0" customHeight="1">
-      <c r="A30" s="27"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="29" t="s">
-        <v>63</v>
-      </c>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27"/>
-      <c r="O30" s="27"/>
-      <c r="P30" s="27"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="27"/>
-      <c r="V30" s="27"/>
-      <c r="W30" s="27"/>
-      <c r="X30" s="27"/>
-      <c r="Y30" s="27"/>
-      <c r="Z30" s="27"/>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>So sánh các phương pháp/ thảo luận / kết luận</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13" t="n"/>
+    </row>
+    <row r="28" ht="14.4" customHeight="1">
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>Nhận xét chung của GV_ : 
+- Hoàn thiện report
+- Bổ sung tinh chỉnh models
+- Chỉnh sửa demo
+- Tăng độ chính xác model
+- Khuyến nghị BV lần 1</t>
+        </is>
+      </c>
+      <c r="C28" s="40" t="n"/>
+      <c r="D28" s="40" t="n"/>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>Khuyến nghị của GV Review:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="20" t="n"/>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>Kết quả khuyến nghị</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="n"/>
+      <c r="H30" s="19" t="n"/>
+      <c r="I30" s="19" t="n"/>
+      <c r="J30" s="19" t="n"/>
+      <c r="K30" s="19" t="n"/>
+      <c r="L30" s="19" t="n"/>
+      <c r="M30" s="19" t="n"/>
+      <c r="N30" s="19" t="n"/>
+      <c r="O30" s="19" t="n"/>
+      <c r="P30" s="19" t="n"/>
+      <c r="Q30" s="19" t="n"/>
+      <c r="R30" s="19" t="n"/>
+      <c r="S30" s="19" t="n"/>
+      <c r="T30" s="19" t="n"/>
+      <c r="U30" s="19" t="n"/>
+      <c r="V30" s="19" t="n"/>
+      <c r="W30" s="19" t="n"/>
+      <c r="X30" s="19" t="n"/>
+      <c r="Y30" s="19" t="n"/>
+      <c r="Z30" s="19" t="n"/>
     </row>
     <row r="31" ht="32.25" customHeight="1">
-      <c r="B31" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="C31" s="31"/>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>1/Kết quả KLTN đủ tiêu chuẩn để bảo vệ lần 1</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="n"/>
     </row>
     <row r="32" ht="32.25" customHeight="1">
-      <c r="B32" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" s="31"/>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>2/Cần cập nhật, bổ sung theo những góp ý của GV Review để bảo vệ lần 1</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="n"/>
     </row>
     <row r="33" ht="32.25" customHeight="1">
-      <c r="B33" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="C33" s="31"/>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>3/Kết quả KLTN còn nhiều thiếu sót. Phải bổ sung đầy đủ theo những góp ý và bảo vệ lần 2</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="n"/>
     </row>
     <row r="34" ht="32.25" customHeight="1">
-      <c r="B34" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" s="31"/>
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>4/Kết quả KLTN có những thiếu sót nghiêm trọng, không đáp ứng được tiêu chuẩn của KLTN ngành TTNT. Nhóm nên chấm dứt dự án KLTN</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1"/>
     <row r="36" ht="15.75" customHeight="1"/>
@@ -4492,21 +5336,19 @@
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B17:B21"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B12:B16"/>
     <mergeCell ref="B22:B26"/>
-    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:B16"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="portrait" paperSize="1"/>
 </worksheet>
 </file>
</xml_diff>